<commit_message>
final matrix vs TN comparison data
</commit_message>
<xml_diff>
--- a/diffusion-tn/validation/matrix_vs_tn_memory_n=7.xlsx
+++ b/diffusion-tn/validation/matrix_vs_tn_memory_n=7.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aditya/Desktop/UROPS/mps-fluid-dynamics/diffusion-tn/validation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D9F85A28-D8C4-7E42-BF85-FB1D096D0DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC1DACB9-7763-B840-B20B-7DFF105A17C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="15420" windowHeight="18960" activeTab="2" xr2:uid="{216AEBAE-1D9E-8E4C-BCAE-552C49E81715}"/>
+    <workbookView xWindow="-27320" yWindow="-220" windowWidth="27320" windowHeight="19860" activeTab="1" xr2:uid="{216AEBAE-1D9E-8E4C-BCAE-552C49E81715}"/>
   </bookViews>
   <sheets>
     <sheet name="matrix_vs_tn_memory" sheetId="1" r:id="rId1"/>
-    <sheet name="avg memory per step" sheetId="3" r:id="rId2"/>
+    <sheet name="median memory per step" sheetId="3" r:id="rId2"/>
     <sheet name="setup" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="16">
   <si>
     <t>n</t>
   </si>
@@ -92,22 +92,19 @@
     <t>N=2^n</t>
   </si>
   <si>
-    <t>MPS (s)</t>
-  </si>
-  <si>
-    <t>MPO (s)</t>
-  </si>
-  <si>
-    <t>TN=MPS+MPO (s)</t>
-  </si>
-  <si>
-    <t>Matrix (s)</t>
-  </si>
-  <si>
     <t>Matrix (MB)</t>
   </si>
   <si>
     <t>TN (MB)</t>
+  </si>
+  <si>
+    <t>TN=MPS+MPO (MB)</t>
+  </si>
+  <si>
+    <t>MPO (MB)</t>
+  </si>
+  <si>
+    <t>MPS (MB)</t>
   </si>
 </sst>
 </file>
@@ -785,7 +782,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-GB" sz="1800"/>
-              <a:t>Average memory</a:t>
+              <a:t>Median memory</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-GB" sz="1800" baseline="0"/>
@@ -820,7 +817,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -835,7 +832,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'avg memory per step'!$C$1</c:f>
+              <c:f>'median memory per step'!$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -870,7 +867,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'avg memory per step'!$B$2:$B$5</c:f>
+              <c:f>'median memory per step'!$B$2:$B$5</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="4"/>
@@ -891,7 +888,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'avg memory per step'!$C$2:$C$5</c:f>
+              <c:f>'median memory per step'!$C$2:$C$5</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="4"/>
@@ -922,7 +919,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'avg memory per step'!$D$1</c:f>
+              <c:f>'median memory per step'!$D$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -957,7 +954,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'avg memory per step'!$B$2:$B$5</c:f>
+              <c:f>'median memory per step'!$B$2:$B$5</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="4"/>
@@ -978,7 +975,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'avg memory per step'!$D$2:$D$8</c:f>
+              <c:f>'median memory per step'!$D$2:$D$8</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="7"/>
@@ -1101,7 +1098,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1188,7 +1185,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-GB" sz="1400"/>
-                  <a:t>Average memory allocated per</a:t>
+                  <a:t>Median memory allocated per</a:t>
                 </a:r>
                 <a:r>
                   <a:rPr lang="en-GB" sz="1400" baseline="0"/>
@@ -1385,7 +1382,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1800"/>
-              <a:t>Average memory allocated per TN step</a:t>
+              <a:t>Median memory allocated per TN step</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-US" sz="1800" baseline="0"/>
@@ -1435,7 +1432,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'avg memory per step'!$D$1</c:f>
+              <c:f>'median memory per step'!$D$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1446,9 +1443,7 @@
           </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -1468,39 +1463,89 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-7.8490257757354881E-2"/>
+                  <c:y val="0.30344745576985499"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'avg memory per step'!$B$2:$B$8</c:f>
+              <c:f>'median memory per step'!$A$2:$A$8</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>16</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>32</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>64</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>128</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>256</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>512</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1024</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'avg memory per step'!$D$2:$D$8</c:f>
+              <c:f>'median memory per step'!$D$2:$D$8</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="7"/>
@@ -1550,8 +1595,8 @@
         <c:axId val="363503039"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="1040"/>
-          <c:min val="0"/>
+          <c:max val="10"/>
+          <c:min val="4"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -1604,11 +1649,19 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-GB" sz="1400"/>
-                  <a:t>System size,</a:t>
+                  <a:t>System size parameter</a:t>
                 </a:r>
                 <a:r>
                   <a:rPr lang="en-GB" sz="1400" baseline="0"/>
-                  <a:t> N</a:t>
+                  <a:t> n</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" sz="1400"/>
+                  <a:t>,</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" sz="1400" baseline="0"/>
+                  <a:t> N=2^n</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-GB" sz="1400"/>
               </a:p>
@@ -1639,7 +1692,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1726,7 +1779,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-GB" sz="1400"/>
-                  <a:t>Average memory allocated</a:t>
+                  <a:t>Median memory allocated</a:t>
                 </a:r>
                 <a:r>
                   <a:rPr lang="en-GB" sz="1400" baseline="0"/>
@@ -1761,7 +1814,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1893,11 +1946,11 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-GB" sz="1800"/>
-              <a:t>Memory Allocated for TN Setup</a:t>
+              <a:t>Memory Allocated for Matrix</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-GB" sz="1800" baseline="0"/>
-              <a:t> vs System size N</a:t>
+              <a:t> vs TN Setup</a:t>
             </a:r>
             <a:endParaRPr lang="en-GB" sz="1800"/>
           </a:p>
@@ -1928,7 +1981,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1947,7 +2000,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>TN=MPS+MPO (s)</c:v>
+                  <c:v>TN=MPS+MPO (MB)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2052,7 +2105,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Matrix (s)</c:v>
+                  <c:v>Matrix (MB)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2146,7 +2199,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1040"/>
-          <c:min val="-"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -2320,7 +2373,7 @@
                 </a:r>
                 <a:r>
                   <a:rPr lang="en-GB" sz="1400" baseline="0"/>
-                  <a:t> TN setup (MB)</a:t>
+                  <a:t> setup (MB)</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-GB" sz="1400"/>
               </a:p>
@@ -2351,7 +2404,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -2404,6 +2457,37 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -4279,16 +4363,16 @@
     <tableColumn id="6" xr3:uid="{A6227CEB-468C-774D-BE6C-7785C4BE9FBA}" name="N=2^n" dataDxfId="9">
       <calculatedColumnFormula>2^Table3[[#This Row],[n]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{FE9B16D4-41A8-4846-9B8C-C9EDA4736E45}" name="MPS (s)" dataDxfId="7">
+    <tableColumn id="3" xr3:uid="{FE9B16D4-41A8-4846-9B8C-C9EDA4736E45}" name="MPS (MB)" dataDxfId="8">
       <calculatedColumnFormula array="1">MEDIAN(_xlfn._xlws.FILTER(matrix_vs_tn_memory!H:H,matrix_vs_tn_memory!$A:$A=$A2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{576FA662-75CD-9642-8887-7CFA93142E38}" name="MPO (s)" dataDxfId="6">
+    <tableColumn id="4" xr3:uid="{576FA662-75CD-9642-8887-7CFA93142E38}" name="MPO (MB)" dataDxfId="7">
       <calculatedColumnFormula array="1">MEDIAN(_xlfn._xlws.FILTER(matrix_vs_tn_memory!I:I,matrix_vs_tn_memory!$A:$A=$A2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{611C756E-7B98-C443-98FE-2C9CB9368A98}" name="TN=MPS+MPO (s)" dataDxfId="8">
+    <tableColumn id="5" xr3:uid="{611C756E-7B98-C443-98FE-2C9CB9368A98}" name="TN=MPS+MPO (MB)" dataDxfId="6">
       <calculatedColumnFormula>C2+D2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67701714-7385-874D-9C30-EDD82DDB78D6}" name="Matrix (s)" dataDxfId="5">
+    <tableColumn id="2" xr3:uid="{67701714-7385-874D-9C30-EDD82DDB78D6}" name="Matrix (MB)" dataDxfId="5">
       <calculatedColumnFormula array="1">MEDIAN(_xlfn._xlws.FILTER(matrix_vs_tn_memory!G:G,matrix_vs_tn_memory!$A:$A=$A2))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -24979,10 +25063,10 @@
         <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -25117,16 +25201,16 @@
         <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E1" t="s">
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>